<commit_message>
minimale fixes für die Präsi
</commit_message>
<xml_diff>
--- a/References.xlsx
+++ b/References.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="DieseArbeitsmappe"/>
   <bookViews>
-    <workbookView windowWidth="14880" windowHeight="11655" firstSheet="1" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12180" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Import" sheetId="30" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="278">
   <si>
     <t>@article{example2024,   title = {A Reference Example},   journal = {Journal of Examples},   publisher = {Example Press},   author = {Doe, Jane},   year = {2024},   month = aug,   pages = {185–209} }</t>
   </si>
@@ -2781,6 +2781,21 @@
 </t>
   </si>
   <si>
+    <t>@incollection{HagerHasselhorn2000,
+  author    = {Hager, Willi and Hasselhorn, Marcus},
+  title     = {{Psychologische Interventionsmaßnahmen: Was sollen sie bewirken können?}},
+  booktitle = {{Evaluation psychologischer Interventionsmaßnahmen}},
+  editor    = {Hager, Willi and Patry, Jean-Luc and Brezing, Hermann},
+  year      = {2000},
+  pages     = {41--85},
+  publisher = {Huber},
+  address   = {Bern}
+}</t>
+  </si>
+  <si>
+    <t>definition</t>
+  </si>
+  <si>
     <t>Bibtex templates</t>
   </si>
   <si>
@@ -26958,14 +26973,16 @@
       <c r="I174" s="26"/>
     </row>
     <row r="175" ht="36" customHeight="1" spans="1:11">
-      <c r="A175" s="19"/>
+      <c r="A175" s="19" t="s">
+        <v>233</v>
+      </c>
       <c r="B175" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@HagerHasselhorn2000</v>
       </c>
       <c r="C175" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@HagerHasselhorn2000]</v>
       </c>
       <c r="D175" s="22" t="str">
         <f t="shared" si="28"/>
@@ -26977,17 +26994,19 @@
       </c>
       <c r="F175" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>{Evaluation psychologischer Interventionsmaßnahmen}</v>
       </c>
       <c r="G175" s="24" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="H175" s="25" t="str">
+      <c r="H175" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="I175" s="26"/>
+        <v>46125.5496643518</v>
+      </c>
+      <c r="I175" s="26" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="176" ht="36" customHeight="1" spans="1:11">
       <c r="A176" s="19"/>
@@ -37342,176 +37361,176 @@
   <sheetData>
     <row r="1" ht="47.25" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="72.75" customHeight="1" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" ht="180" customHeight="1" spans="1:3">
       <c r="A5" s="7" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" ht="210" customHeight="1" spans="1:3">
       <c r="A6" s="7" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" ht="210" customHeight="1" spans="1:3">
       <c r="A7" s="7" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" ht="150" customHeight="1" spans="1:3">
       <c r="A8" s="7" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" ht="255" customHeight="1" spans="1:3">
       <c r="A9" s="7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" ht="255" customHeight="1" spans="1:3">
       <c r="A10" s="7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" ht="285" customHeight="1" spans="1:3">
       <c r="A11" s="7" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" ht="285" customHeight="1" spans="1:3">
       <c r="A12" s="7" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" ht="255" customHeight="1" spans="1:3">
       <c r="A13" s="7" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" ht="165" customHeight="1" spans="1:3">
       <c r="A14" s="7" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" ht="165" customHeight="1" spans="1:3">
       <c r="A15" s="7" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16" ht="165" customHeight="1" spans="1:3">
       <c r="A16" s="7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="17" ht="225" customHeight="1" spans="1:3">
       <c r="A17" s="7" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="18" ht="180" customHeight="1" spans="1:3">
       <c r="A18" s="7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="19" ht="105" customHeight="1" spans="1:3">
       <c r="A19" s="7" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" ht="120" customHeight="1" spans="1:3">
       <c r="A20" s="7" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" ht="135" customHeight="1" spans="1:3">
       <c r="A21" s="7" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update für die zweite Präsentation
</commit_message>
<xml_diff>
--- a/References.xlsx
+++ b/References.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="284">
   <si>
     <t>@article{example2024,   title = {A Reference Example},   journal = {Journal of Examples},   publisher = {Example Press},   author = {Doe, Jane},   year = {2024},   month = aug,   pages = {185–209} }</t>
   </si>
@@ -2796,6 +2796,78 @@
     <t>definition</t>
   </si>
   <si>
+    <t>@book{sedlmeier_forschungsmethoden_2018,
+ author = {Sedlmeier, Peter and Renkewitz, Frank},
+ title = {Forschungsmethoden und Statistik für Psychologen und Sozialwissenschaftler},
+ edition = {3., aktualisierte und erweiterte Auflage},
+ year = {2018},
+ publisher = {Pearson Deutschland GmbH},
+ address = {Hallbergmoos},
+ isbn = {978-3-86894-321-4}
+}</t>
+  </si>
+  <si>
+    <t>@article{PANAS,
+  doi = {10.6102/ZIS242},
+  url = {http://zis.gesis.org/DoiId/zis242},
+  author = {Breyer,  B. and Bluemke,  M.},
+  keywords = {Affektivit\"{a}t,  Wohlbefinden,  Gef\"{u}hl,  Emotion},
+  language = {de},
+  title = {Deutsche Version der Positive and Negative Affect Schedule PANAS (GESIS Panel)},
+  journal = {Zusammenstellung sozialwissenschaftlicher Items und Skalen (ZIS)},
+  publisher = {ZIS - GESIS Leibniz Institute for the Social Sciences},
+  year = {2016},
+  copyright = {Nutzungsbedingungen: Alle in ZIS dokumentierten Erhebungsinstrumente d\"{u}rfen kostenfrei f\"{u}r nicht-kommerzielle Forschungszwecke verwendet werden.Bei einem Einsatz f\"{u}r andere Zwecke oder in einer anderen als der hier dokumentierten Form ist das Einverst\"{a}ndnis der Autoren bzw. Autorinnen einzuholen. In allen resultierenden Arbeiten und Publikationen ist die ZIS-Dokumentation als Quelle anzugeben.}
+}</t>
+  </si>
+  <si>
+    <t>@article{mcauley_long-term_1993,
+ author = {McAuley, Edward and Lox, Curt and Duncan, Terry E.},
+ title = {Long-term maintenance of exercise, self-efficacy, and physiological change in older adults},
+ journal = {Journal of Gerontology: Psychological Sciences},
+ volume = {48},
+ number = {4},
+ pages = {P218-P224},
+ year = {1993},
+ publisher = {The Gerontological Society of America}
+}</t>
+  </si>
+  <si>
+    <t>@misc{grossheinrich_panas-c-p_2020,
+ author = {Großheinrich, N.},
+ title = {PANAS-C-P: Parent Version of the Positive and Negative Affect Scale for Children - deutsche Fassung},
+ year = {2020},
+ publisher = {ZPID (Leibniz-Institut für Psychologie)},
+ series = {Open Test Archive},
+ address = {Trier},
+ doi = {10.23668/psycharchives.4491},
+ url = {https://www.testarchiv.eu/de/test/9007913}
+}</t>
+  </si>
+  <si>
+    <t>@article{resnick_testing_2000,
+ author = {Resnick, B. and Jenkins, L. S.},
+ title = {Testing the reliability and validity of the Self-Efficacy for Exercise Scale},
+ journal = {Nursing Research},
+ volume = {49},
+ number = {3},
+ pages = {154-159},
+ year = {2000}
+}</t>
+  </si>
+  <si>
+    <t>@article{laurent_measure_1999,
+ author = {Laurent, J. and Catanzaro, S. J. and Joiner, T. E. Jr. and Rudolph, K. D. and Potter, K. I. and Lambert, S. and Osborne, L. and Gathright, T.},
+ title = {A measure of positive and negative affect for children: Scale development and preliminary validation},
+ journal = {Psychological Assessment},
+ volume = {11},
+ number = {3},
+ pages = {326-338},
+ year = {1999},
+ doi = {10.1037/1040-3590.11.3.326}
+}</t>
+  </si>
+  <si>
     <t>Bibtex templates</t>
   </si>
   <si>
@@ -27009,196 +27081,214 @@
       </c>
     </row>
     <row r="176" ht="36" customHeight="1" spans="1:11">
-      <c r="A176" s="19"/>
+      <c r="A176" s="19" t="s">
+        <v>235</v>
+      </c>
       <c r="B176" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@sedlmeier_forschungsmethoden_2018</v>
       </c>
       <c r="C176" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@sedlmeier_forschungsmethoden_2018]</v>
       </c>
       <c r="D176" s="22" t="str">
         <f t="shared" si="28"/>
-        <v/>
+        <v>2018</v>
       </c>
       <c r="E176" s="22" t="str">
         <f t="shared" si="29"/>
-        <v/>
+        <v>Sedlmeier, Peter and Renkewitz, Frank</v>
       </c>
       <c r="F176" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>Forschungsmethoden und Statistik für Psychologen und Sozialwissenschaftler</v>
       </c>
       <c r="G176" s="24" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="H176" s="25" t="str">
+      <c r="H176" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
+        <v>46129.4323032407</v>
       </c>
       <c r="I176" s="26"/>
     </row>
     <row r="177" ht="36" customHeight="1" spans="1:9">
-      <c r="A177" s="19"/>
+      <c r="A177" s="19" t="s">
+        <v>236</v>
+      </c>
       <c r="B177" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@PANAS</v>
       </c>
       <c r="C177" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@PANAS]</v>
       </c>
       <c r="D177" s="22" t="str">
         <f t="shared" si="28"/>
-        <v/>
+        <v>2016</v>
       </c>
       <c r="E177" s="22" t="str">
         <f t="shared" si="29"/>
-        <v/>
+        <v>Breyer,  B. and Bluemke,  M.</v>
       </c>
       <c r="F177" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>Deutsche Version der Positive and Negative Affect Schedule PANAS (GESIS Panel)</v>
       </c>
       <c r="G177" s="24" t="str">
         <f t="shared" si="31"/>
-        <v/>
-      </c>
-      <c r="H177" s="25" t="str">
+        <v>https://doi.org/10.6102/ZIS242</v>
+      </c>
+      <c r="H177" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
+        <v>46129.6597453704</v>
       </c>
       <c r="I177" s="26"/>
     </row>
     <row r="178" ht="36" customHeight="1" spans="1:9">
-      <c r="A178" s="19"/>
+      <c r="A178" s="19" t="s">
+        <v>237</v>
+      </c>
       <c r="B178" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@mcauley_long-term_1993</v>
       </c>
       <c r="C178" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@mcauley_long-term_1993]</v>
       </c>
       <c r="D178" s="22" t="str">
         <f t="shared" si="28"/>
-        <v/>
+        <v>1993</v>
       </c>
       <c r="E178" s="22" t="str">
         <f t="shared" si="29"/>
-        <v/>
+        <v>McAuley, Edward and Lox, Curt and Duncan, Terry E.</v>
       </c>
       <c r="F178" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>Long-term maintenance of exercise, self-efficacy, and physiological change in older adults</v>
       </c>
       <c r="G178" s="24" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="H178" s="25" t="str">
+      <c r="H178" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
+        <v>46129.6695833333</v>
       </c>
       <c r="I178" s="26"/>
     </row>
     <row r="179" ht="36" customHeight="1" spans="1:9">
-      <c r="A179" s="19"/>
+      <c r="A179" s="19" t="s">
+        <v>238</v>
+      </c>
       <c r="B179" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@grossheinrich_panas-c-p_2020</v>
       </c>
       <c r="C179" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@grossheinrich_panas-c-p_2020]</v>
       </c>
       <c r="D179" s="22" t="str">
         <f t="shared" si="28"/>
-        <v/>
+        <v>2020</v>
       </c>
       <c r="E179" s="22" t="str">
         <f t="shared" si="29"/>
-        <v/>
+        <v>Großheinrich, N.</v>
       </c>
       <c r="F179" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>PANAS-C-P: Parent Version of the Positive and Negative Affect Scale for Children - deutsche Fassung</v>
       </c>
       <c r="G179" s="24" t="str">
         <f t="shared" si="31"/>
-        <v/>
-      </c>
-      <c r="H179" s="25" t="str">
+        <v>https://doi.org/10.23668/psycharchives.4491</v>
+      </c>
+      <c r="H179" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="I179" s="26"/>
+        <v>46131.7777199074</v>
+      </c>
+      <c r="I179" s="26" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="180" ht="36" customHeight="1" spans="1:9">
-      <c r="A180" s="19"/>
+      <c r="A180" s="19" t="s">
+        <v>239</v>
+      </c>
       <c r="B180" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@resnick_testing_2000</v>
       </c>
       <c r="C180" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@resnick_testing_2000]</v>
       </c>
       <c r="D180" s="22" t="str">
         <f t="shared" si="28"/>
-        <v/>
+        <v>2000</v>
       </c>
       <c r="E180" s="22" t="str">
         <f t="shared" si="29"/>
-        <v/>
+        <v>Resnick, B. and Jenkins, L. S.</v>
       </c>
       <c r="F180" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>Testing the reliability and validity of the Self-Efficacy for Exercise Scale</v>
       </c>
       <c r="G180" s="24" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="H180" s="25" t="str">
+      <c r="H180" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="I180" s="26"/>
+        <v>46131.7778472222</v>
+      </c>
+      <c r="I180" s="26" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="181" ht="36" customHeight="1" spans="1:9">
-      <c r="A181" s="19"/>
+      <c r="A181" s="19" t="s">
+        <v>240</v>
+      </c>
       <c r="B181" s="20" t="str">
         <f t="shared" si="26"/>
-        <v/>
+        <v>@laurent_measure_1999</v>
       </c>
       <c r="C181" s="21" t="str">
         <f t="shared" si="27"/>
-        <v>[]</v>
+        <v>[@laurent_measure_1999]</v>
       </c>
       <c r="D181" s="22" t="str">
         <f t="shared" si="28"/>
-        <v/>
+        <v>1999</v>
       </c>
       <c r="E181" s="22" t="str">
         <f t="shared" si="29"/>
-        <v/>
+        <v>Laurent, J. and Catanzaro, S. J. and Joiner, T. E. Jr. and Rudolph, K. D. and Potter, K. I. and Lambert, S. and Osborne, L. and Gathright, T.</v>
       </c>
       <c r="F181" s="23" t="str">
         <f t="shared" si="30"/>
-        <v/>
+        <v>A measure of positive and negative affect for children: Scale development and preliminary validation</v>
       </c>
       <c r="G181" s="24" t="str">
         <f t="shared" si="31"/>
-        <v/>
-      </c>
-      <c r="H181" s="25" t="str">
+        <v>https://doi.org/10.1037/1040-3590.11.3.326</v>
+      </c>
+      <c r="H181" s="25">
         <f ca="1" t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="I181" s="26"/>
+        <v>46131.7779398148</v>
+      </c>
+      <c r="I181" s="26" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="182" ht="36" customHeight="1" spans="1:9">
       <c r="A182" s="19"/>
@@ -37361,176 +37451,176 @@
   <sheetData>
     <row r="1" ht="47.25" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="72.75" customHeight="1" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" ht="180" customHeight="1" spans="1:3">
       <c r="A5" s="7" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" ht="210" customHeight="1" spans="1:3">
       <c r="A6" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" ht="210" customHeight="1" spans="1:3">
       <c r="A7" s="7" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" ht="150" customHeight="1" spans="1:3">
       <c r="A8" s="7" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" ht="255" customHeight="1" spans="1:3">
       <c r="A9" s="7" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" ht="255" customHeight="1" spans="1:3">
       <c r="A10" s="7" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" ht="285" customHeight="1" spans="1:3">
       <c r="A11" s="7" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" ht="285" customHeight="1" spans="1:3">
       <c r="A12" s="7" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" ht="255" customHeight="1" spans="1:3">
       <c r="A13" s="7" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" ht="165" customHeight="1" spans="1:3">
       <c r="A14" s="7" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" ht="165" customHeight="1" spans="1:3">
       <c r="A15" s="7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="16" ht="165" customHeight="1" spans="1:3">
       <c r="A16" s="7" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" ht="225" customHeight="1" spans="1:3">
       <c r="A17" s="7" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="18" ht="180" customHeight="1" spans="1:3">
       <c r="A18" s="7" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" ht="105" customHeight="1" spans="1:3">
       <c r="A19" s="7" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="20" ht="120" customHeight="1" spans="1:3">
       <c r="A20" s="7" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21" ht="135" customHeight="1" spans="1:3">
       <c r="A21" s="7" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
R Skript für LV6
</commit_message>
<xml_diff>
--- a/References.xlsx
+++ b/References.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="290">
   <si>
     <t>@article{example2024,   title = {A Reference Example},   journal = {Journal of Examples},   publisher = {Example Press},   author = {Doe, Jane},   year = {2024},   month = aug,   pages = {185–209} }</t>
   </si>
@@ -2924,6 +2924,34 @@
 }</t>
   </si>
   <si>
+    <t>@article{Domin2021,
+  title = {Smartphone-Based Interventions for Physical Activity Promotion: Scoping Review of the Evidence Over the Last 10 Years},
+  volume = {9},
+  ISSN = {2291-5222},
+  url = {http://dx.doi.org/10.2196/24308},
+  DOI = {10.2196/24308},
+  number = {7},
+  journal = {JMIR mHealth and uHealth},
+  publisher = {JMIR Publications Inc.},
+  author = {Domin,  Alex and Spruijt-Metz,  Donna and Theisen,  Daniel and Ouzzahra,  Yacine and V\"{o}gele,  Claus},
+  year = {2021},
+  month = July,
+  pages = {e24308}
+}</t>
+  </si>
+  <si>
+    <t>@article{Michie2013,
+  author = {Michie, Susan and Richardson, Michelle and Johnston, Marie and Abraham, Charles and Francis, Jill and Hardeman, Wendy and Eccles, Martin P. and Cane, James and Wood, Caroline E.},
+  title = {The behavior change technique taxonomy (v1) of 93 hierarchically clustered techniques: building an international consensus for the reporting of behavior change interventions},
+  journal = {Annals of Behavioral Medicine},
+  volume = {46},
+  number = {1},
+  pages = {81--95},
+  year = {2013},
+  doi = {10.1007/s12160-013-9486-6}
+}</t>
+  </si>
+  <si>
     <t>Bibtex templates</t>
   </si>
   <si>
@@ -27483,66 +27511,70 @@
       <c r="I185" s="26"/>
     </row>
     <row r="186" ht="36" customHeight="1" spans="1:9">
-      <c r="A186" s="19"/>
+      <c r="A186" s="19" t="s">
+        <v>245</v>
+      </c>
       <c r="B186" s="20" t="str">
         <f t="shared" si="38"/>
-        <v/>
+        <v>@Domin2021</v>
       </c>
       <c r="C186" s="21" t="str">
         <f t="shared" si="39"/>
-        <v>[]</v>
+        <v>[@Domin2021]</v>
       </c>
       <c r="D186" s="22" t="str">
         <f t="shared" si="33"/>
-        <v/>
+        <v>2021</v>
       </c>
       <c r="E186" s="22" t="str">
         <f t="shared" si="34"/>
-        <v/>
+        <v>Domin,  Alex and Spruijt-Metz,  Donna and Theisen,  Daniel and Ouzzahra,  Yacine and V\"{o</v>
       </c>
       <c r="F186" s="23" t="str">
         <f t="shared" si="35"/>
-        <v/>
+        <v>Smartphone-Based Interventions for Physical Activity Promotion: Scoping Review of the Evidence Over the Last 10 Years</v>
       </c>
       <c r="G186" s="24" t="str">
         <f t="shared" si="36"/>
-        <v/>
-      </c>
-      <c r="H186" s="25" t="str">
+        <v>https://doi.org/10.2196/24308</v>
+      </c>
+      <c r="H186" s="25">
         <f ca="1" t="shared" si="37"/>
-        <v/>
+        <v>46146.7011574074</v>
       </c>
       <c r="I186" s="26"/>
     </row>
     <row r="187" ht="36" customHeight="1" spans="1:9">
-      <c r="A187" s="19"/>
+      <c r="A187" s="19" t="s">
+        <v>246</v>
+      </c>
       <c r="B187" s="20" t="str">
         <f t="shared" si="38"/>
-        <v/>
+        <v>@Michie2013</v>
       </c>
       <c r="C187" s="21" t="str">
         <f t="shared" si="39"/>
-        <v>[]</v>
+        <v>[@Michie2013]</v>
       </c>
       <c r="D187" s="22" t="str">
         <f t="shared" si="33"/>
-        <v/>
+        <v>2013</v>
       </c>
       <c r="E187" s="22" t="str">
         <f t="shared" si="34"/>
-        <v/>
+        <v>Michie, Susan and Richardson, Michelle and Johnston, Marie and Abraham, Charles and Francis, Jill and Hardeman, Wendy and Eccles, Martin P. and Cane, James and Wood, Caroline E.</v>
       </c>
       <c r="F187" s="23" t="str">
         <f t="shared" si="35"/>
-        <v/>
+        <v>The behavior change technique taxonomy (v1) of 93 hierarchically clustered techniques: building an international consensus for the reporting of behavior change interventions</v>
       </c>
       <c r="G187" s="24" t="str">
         <f t="shared" si="36"/>
-        <v/>
-      </c>
-      <c r="H187" s="25" t="str">
+        <v>https://doi.org/10.1007/s12160-013-9486-6</v>
+      </c>
+      <c r="H187" s="25">
         <f ca="1" t="shared" si="37"/>
-        <v/>
+        <v>46146.70125</v>
       </c>
       <c r="I187" s="26"/>
     </row>
@@ -37515,176 +37547,176 @@
   <sheetData>
     <row r="1" ht="47.25" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="72.75" customHeight="1" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" ht="180" customHeight="1" spans="1:3">
       <c r="A5" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" ht="210" customHeight="1" spans="1:3">
       <c r="A6" s="7" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" ht="210" customHeight="1" spans="1:3">
       <c r="A7" s="7" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" ht="150" customHeight="1" spans="1:3">
       <c r="A8" s="7" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" ht="255" customHeight="1" spans="1:3">
       <c r="A9" s="7" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" ht="255" customHeight="1" spans="1:3">
       <c r="A10" s="7" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" ht="285" customHeight="1" spans="1:3">
       <c r="A11" s="7" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" ht="285" customHeight="1" spans="1:3">
       <c r="A12" s="7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" ht="255" customHeight="1" spans="1:3">
       <c r="A13" s="7" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" ht="165" customHeight="1" spans="1:3">
       <c r="A14" s="7" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15" ht="165" customHeight="1" spans="1:3">
       <c r="A15" s="7" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" ht="165" customHeight="1" spans="1:3">
       <c r="A16" s="7" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" ht="225" customHeight="1" spans="1:3">
       <c r="A17" s="7" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" ht="180" customHeight="1" spans="1:3">
       <c r="A18" s="7" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="19" ht="105" customHeight="1" spans="1:3">
       <c r="A19" s="7" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" ht="120" customHeight="1" spans="1:3">
       <c r="A20" s="7" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" ht="135" customHeight="1" spans="1:3">
       <c r="A21" s="7" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>